<commit_message>
METING_BUS: bus-connected temperature sensors emit a cable despite having no AI
NW-sens sensors (NSB8BTN...) report over the data bus and occupy no analogue
input, but Erco still runs a cable to them. _ok() rejected METING_PASSIEF
without AI, so ten rows in 2195-06 silently produced nothing.

- 1_Synoniemen: patterns 'nsb8btn' and 'nw-sens' -> METING_BUS, prio 70
  (above 'temperatuur' at 65)
- 2_Kabelkeuze: new METING_BUS row. B2CA value from the 2195-06 manual,
  CCA value copied from METING_ACTIEF - both PROVISIONAL, pending Rick
- rules.py: METING_BUS added to sig_priority ahead of METING_PASSIEF
- rules.py: _ok() exempts METING_BUS from the AI requirement

The AI check is retained for everything else - it is what correctly declines
the Muurbeugel RVS bracket rows.

2195-06: 96 -> 106 cables, 46 -> 36 flags. Merge gate 3/3.
</commit_message>
<xml_diff>
--- a/config/kabelconfig.xlsx
+++ b/config/kabelconfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\io2cable\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDF9A88-F117-474E-AFBD-AF6781ADFF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{162ED4B9-50D7-4AF3-B783-E7B04CC1E965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="28650" windowHeight="16950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17430" yWindow="7035" windowWidth="23010" windowHeight="13650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0_Parameters" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="447">
   <si>
     <t>Step 0 — fill in per project BEFORE generation. Yellow fields are mandatory. Values in 'opties' (geen/erco/derden) are literal keys read by the engine — keep them as-is.</t>
   </si>
@@ -1358,7 +1358,28 @@
     <t>DRAK</t>
   </si>
   <si>
-    <t>B2CA</t>
+    <t>CCA</t>
+  </si>
+  <si>
+    <t>nsb8btn</t>
+  </si>
+  <si>
+    <t>nw-sens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	NW-sens bus temperature sensor; no AI by design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	same, matched on omschrijving (OCR-safe alternative)</t>
+  </si>
+  <si>
+    <t>DRAK SIGK 1X4X0,8 B2CA HA500</t>
+  </si>
+  <si>
+    <t>B2CA HA500	bus-connected temp sensor, no AI by design; B2CA value from 2195-06 manual — UNCONFIRMED</t>
+  </si>
+  <si>
+    <t>METING_BUS</t>
   </si>
 </sst>
 </file>
@@ -1949,7 +1970,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D120"/>
+  <dimension ref="A1:D122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -3547,6 +3568,34 @@
         <v>275</v>
       </c>
     </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>440</v>
+      </c>
+      <c r="B121" t="s">
+        <v>446</v>
+      </c>
+      <c r="C121">
+        <v>70</v>
+      </c>
+      <c r="D121" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>441</v>
+      </c>
+      <c r="B122" t="s">
+        <v>446</v>
+      </c>
+      <c r="C122">
+        <v>70</v>
+      </c>
+      <c r="D122" t="s">
+        <v>443</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3554,7 +3603,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -4245,6 +4294,20 @@
       </c>
       <c r="D51" t="s">
         <v>363</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>446</v>
+      </c>
+      <c r="B52" t="s">
+        <v>288</v>
+      </c>
+      <c r="C52" t="s">
+        <v>444</v>
+      </c>
+      <c r="D52" t="s">
+        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated header_aliases in ingest.py
</commit_message>
<xml_diff>
--- a/config/kabelconfig.xlsx
+++ b/config/kabelconfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\io2cable\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{162ED4B9-50D7-4AF3-B783-E7B04CC1E965}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197AF570-5A49-4F63-8B30-C6A0E4847FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17430" yWindow="7035" windowWidth="23010" windowHeight="13650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="77070" windowHeight="21150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0_Parameters" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="468">
   <si>
     <t>Step 0 — fill in per project BEFORE generation. Yellow fields are mandatory. Values in 'opties' (geen/erco/derden) are literal keys read by the engine — keep them as-is.</t>
   </si>
@@ -917,9 +917,6 @@
     <t>METER_VOEDING_24V</t>
   </si>
   <si>
-    <t>JOBA STUURSTR HHJZ 3X1 MT</t>
-  </si>
-  <si>
     <t>separate feed cable energy meter — CCA per Boerhaave (3X1), B2CA per Duitslandlaan (5X1)</t>
   </si>
   <si>
@@ -962,9 +959,6 @@
     <t>run/fault/control</t>
   </si>
   <si>
-    <t>JOBA STUURSTR HHJZ 7X1 MT</t>
-  </si>
-  <si>
     <t>throttle valve open/close + feedback (Boerhaave CCA validated)</t>
   </si>
   <si>
@@ -989,9 +983,6 @@
     <t>FLOWMETER_TSA</t>
   </si>
   <si>
-    <t>JOBA ST.STR B2CA HCHOZ 6X0,8 MT</t>
-  </si>
-  <si>
     <t>flowmeter TSA (dict: TSA gebouwzijde, 6x0,8)</t>
   </si>
   <si>
@@ -1004,18 +995,12 @@
     <t>warmtewiel motor feed (dict: Luchtbehandeling 1, 3g1,5)</t>
   </si>
   <si>
-    <t>JOBA ST.STR B2CA AFG 3X2X0,8 MT</t>
-  </si>
-  <si>
     <t>warmtewiel vrijgave/storing + sturing 0-10V bundled (dict: 3x2x0,8)</t>
   </si>
   <si>
     <t>DRAK CCA GY 4X0,8 MT</t>
   </si>
   <si>
-    <t>JOBA ST.STR B2CA HCHOZ 4X0,8 MT</t>
-  </si>
-  <si>
     <t>vorstbeveiligings thermostaat (dict: 4x0,8)</t>
   </si>
   <si>
@@ -1025,12 +1010,6 @@
     <t>maximaal thermostaat (dict: Losse componenten, 4x0,8)</t>
   </si>
   <si>
-    <t>DRAK SIGK CCA 2X2X0,8 MT</t>
-  </si>
-  <si>
-    <t>JOBA ST.STR B2CA HCHJZ 2X2X0,8 MT</t>
-  </si>
-  <si>
     <t>stoombevochtiger 0-10V (dict: 2x2x0,8)</t>
   </si>
   <si>
@@ -1067,9 +1046,6 @@
     <t>urgent/niet urgent alarm (dict: Onderstation algemeen, 4x0,8)</t>
   </si>
   <si>
-    <t>JOBA STUURSTR HHJZ 10X1 MT</t>
-  </si>
-  <si>
     <t>brandventilatieschakeling (dict CCA: 6x0,8; Tilburg B2CA: 10X1 -- observed exception)</t>
   </si>
   <si>
@@ -1100,9 +1076,6 @@
     <t>weerstation voeding (dict: Losse componenten, 4x0,8)</t>
   </si>
   <si>
-    <t>DRAK SIGK CCA 1X2X0,64 MT</t>
-  </si>
-  <si>
     <t>weerstation modbus (dict: 1x2x0,64)</t>
   </si>
   <si>
@@ -1358,9 +1331,6 @@
     <t>DRAK</t>
   </si>
   <si>
-    <t>CCA</t>
-  </si>
-  <si>
     <t>nsb8btn</t>
   </si>
   <si>
@@ -1373,20 +1343,113 @@
     <t xml:space="preserve">	same, matched on omschrijving (OCR-safe alternative)</t>
   </si>
   <si>
-    <t>DRAK SIGK 1X4X0,8 B2CA HA500</t>
-  </si>
-  <si>
     <t>B2CA HA500	bus-connected temp sensor, no AI by design; B2CA value from 2195-06 manual — UNCONFIRMED</t>
   </si>
   <si>
     <t>METING_BUS</t>
+  </si>
+  <si>
+    <t>B2CA</t>
+  </si>
+  <si>
+    <t>DRAK HULT CCA 7G1,5 HA500</t>
+  </si>
+  <si>
+    <t>DRAK SIGK AFG CCA 4X2X0,8 MT</t>
+  </si>
+  <si>
+    <t>change this to modbus BMS Cable 2x2x24AWG - R1319</t>
+  </si>
+  <si>
+    <t>BMS Cable 2x2x24AWG - R1319 -  B2ca s1,d0,a1 Violet HA500</t>
+  </si>
+  <si>
+    <t>JOBA ST.STR B2CA HCHJZ 12X1 MT</t>
+  </si>
+  <si>
+    <t>kabel_B2CA_DRAK</t>
+  </si>
+  <si>
+    <t>DRAK SIGK B2CA 1X2X0,8 2501 MT</t>
+  </si>
+  <si>
+    <t>DRAK B2CA GY 2X0,8 MT</t>
+  </si>
+  <si>
+    <t>RAK SIGN KAB B2CA 4X0,8 HA500</t>
+  </si>
+  <si>
+    <t>DRAK SIGK B2CA 1X4X0,8 2502Q MT</t>
+  </si>
+  <si>
+    <t>DRAK B2CA GY 6X0,8 MT</t>
+  </si>
+  <si>
+    <t>DRAK B2CA GY 8X0,8 MT</t>
+  </si>
+  <si>
+    <t>DRAK SIGK AFG B2CA 4X2X0,8 MT</t>
+  </si>
+  <si>
+    <t>DRAK SIGK AFG B2CA 3X2X0,8 MT</t>
+  </si>
+  <si>
+    <t>DRAK HULT B2CA 7G1,5 HA500</t>
+  </si>
+  <si>
+    <t>DRAK HULT B2CA 3G2,5 HA500</t>
+  </si>
+  <si>
+    <t>DRAK HULT B2CA 5G1,5 HA500</t>
+  </si>
+  <si>
+    <t>DRAK HULT B2CA 3G1,5 HA500</t>
+  </si>
+  <si>
+    <t>DRAK B2CA GY 4X0,8 MT</t>
+  </si>
+  <si>
+    <t>kabel_CCA_JOBA</t>
+  </si>
+  <si>
+    <t>JOBA ST.STR CCA HCHOZ 2X1 MT</t>
+  </si>
+  <si>
+    <t>JOBA ST.STR CCA HCHJZ 5X1 MT</t>
+  </si>
+  <si>
+    <t>JOBA STSTR CCA HCHJZ 7X1 MT</t>
+  </si>
+  <si>
+    <t>JOBA ST.STR CCA HCHJZ 7X1 MT</t>
+  </si>
+  <si>
+    <t>DRAK HULT CCA 3G2,5 MT</t>
+  </si>
+  <si>
+    <t>DRAK HULT CCA 5G1,5 MT</t>
+  </si>
+  <si>
+    <t>DRAK HULT CCA 3G1,5 MT</t>
+  </si>
+  <si>
+    <t>BMS Cable 2x2x24AWG - R1319 -  CCA s1,d0,a1 Violet HA500</t>
+  </si>
+  <si>
+    <t>JOBA ST.STR CCA HCHJZ 10X1 MT</t>
+  </si>
+  <si>
+    <t>DRAK SIGK B2CA 1X4X0,8 2501 MT</t>
+  </si>
+  <si>
+    <t>DRAK SIGK CCA 1X4X0,8 2501 MT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1420,6 +1483,24 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1439,7 +1520,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1447,11 +1528,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1461,9 +1558,17 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard 2 3" xfId="1" xr:uid="{8638437D-913E-43F3-9767-5FCE39051AEC}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1844,7 +1949,7 @@
         <v>17</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>18</v>
@@ -1858,7 +1963,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>438</v>
+        <v>429</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>21</v>
@@ -3570,30 +3675,30 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="B121" t="s">
-        <v>446</v>
+        <v>435</v>
       </c>
       <c r="C121">
         <v>70</v>
       </c>
       <c r="D121" t="s">
-        <v>442</v>
+        <v>432</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>441</v>
+        <v>431</v>
       </c>
       <c r="B122" t="s">
-        <v>446</v>
+        <v>435</v>
       </c>
       <c r="C122">
         <v>70</v>
       </c>
       <c r="D122" t="s">
-        <v>443</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -3603,711 +3708,1014 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="3" width="36" customWidth="1"/>
-    <col min="4" max="4" width="52" customWidth="1"/>
+    <col min="2" max="5" width="36" customWidth="1"/>
+    <col min="6" max="6" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>89</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>118</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>108</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>287</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>75</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
         <v>291</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="7" t="s">
+        <v>445</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="F9" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>98</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>112</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>94</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="E13" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>101</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="E14" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>103</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>283</v>
+        <v>445</v>
       </c>
       <c r="C15" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E15" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" t="s">
+        <v>449</v>
+      </c>
+      <c r="C16" t="s">
+        <v>438</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>303</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>159</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="D17" s="3" t="s">
+    </row>
+    <row r="18" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="F18" s="9" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>165</v>
-      </c>
-      <c r="B18" t="s">
-        <v>307</v>
-      </c>
-      <c r="C18" t="s">
-        <v>297</v>
-      </c>
-      <c r="D18" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>174</v>
       </c>
       <c r="B19" t="s">
+        <v>452</v>
+      </c>
+      <c r="C19" t="s">
+        <v>307</v>
+      </c>
+      <c r="D19" t="s">
+        <v>308</v>
+      </c>
+      <c r="E19" t="s">
+        <v>461</v>
+      </c>
+      <c r="F19" t="s">
         <v>309</v>
       </c>
-      <c r="C19" t="s">
-        <v>310</v>
-      </c>
-      <c r="D19" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>181</v>
       </c>
       <c r="B20" t="s">
+        <v>453</v>
+      </c>
+      <c r="C20" t="s">
+        <v>310</v>
+      </c>
+      <c r="D20" t="s">
+        <v>311</v>
+      </c>
+      <c r="E20" t="s">
+        <v>462</v>
+      </c>
+      <c r="F20" t="s">
         <v>312</v>
       </c>
-      <c r="C20" t="s">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>313</v>
       </c>
-      <c r="D20" t="s">
+      <c r="B21" t="s">
+        <v>447</v>
+      </c>
+      <c r="C21" t="s">
+        <v>295</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="F21" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>315</v>
-      </c>
-      <c r="B21" t="s">
-        <v>296</v>
-      </c>
-      <c r="C21" t="s">
-        <v>316</v>
-      </c>
-      <c r="D21" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>185</v>
       </c>
       <c r="B22" t="s">
-        <v>318</v>
+        <v>454</v>
       </c>
       <c r="C22" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="D22" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+        <v>316</v>
+      </c>
+      <c r="E22" t="s">
+        <v>463</v>
+      </c>
+      <c r="F22" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>188</v>
       </c>
       <c r="B23" t="s">
-        <v>305</v>
+        <v>450</v>
       </c>
       <c r="C23" t="s">
-        <v>321</v>
-      </c>
-      <c r="D23" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+        <v>304</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="F23" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>192</v>
       </c>
       <c r="B24" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C24" t="s">
-        <v>324</v>
-      </c>
-      <c r="D24" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F24" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>195</v>
       </c>
       <c r="B25" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C25" t="s">
-        <v>324</v>
-      </c>
-      <c r="D25" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F25" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>198</v>
       </c>
       <c r="B26" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C26" t="s">
-        <v>324</v>
-      </c>
-      <c r="D26" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F26" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>201</v>
       </c>
-      <c r="B27" t="s">
-        <v>328</v>
-      </c>
-      <c r="C27" t="s">
-        <v>329</v>
-      </c>
-      <c r="D27" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B27" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F27" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>203</v>
       </c>
       <c r="B28" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C28" t="s">
+        <v>319</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F28" t="s">
         <v>324</v>
       </c>
-      <c r="D28" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>208</v>
       </c>
       <c r="B29" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C29" t="s">
-        <v>324</v>
-      </c>
-      <c r="D29" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F29" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>211</v>
       </c>
       <c r="B30" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="C30" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="D30" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+        <v>327</v>
+      </c>
+      <c r="E30" t="s">
+        <v>326</v>
+      </c>
+      <c r="F30" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>216</v>
       </c>
-      <c r="B31" t="s">
-        <v>328</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="B31" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F31" t="s">
         <v>329</v>
       </c>
-      <c r="D31" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>219</v>
       </c>
       <c r="B32" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="C32" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="D32" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+        <v>331</v>
+      </c>
+      <c r="E32" t="s">
+        <v>330</v>
+      </c>
+      <c r="F32" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>222</v>
       </c>
       <c r="B33" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C33" t="s">
-        <v>324</v>
-      </c>
-      <c r="D33" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F33" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>225</v>
       </c>
       <c r="B34" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C34" t="s">
-        <v>324</v>
-      </c>
-      <c r="D34" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F34" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>229</v>
       </c>
       <c r="B35" t="s">
-        <v>296</v>
+        <v>447</v>
       </c>
       <c r="C35" t="s">
-        <v>342</v>
-      </c>
-      <c r="D35" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+        <v>295</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="F35" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>232</v>
       </c>
       <c r="B36" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C36" t="s">
-        <v>324</v>
-      </c>
-      <c r="D36" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F36" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>234</v>
       </c>
       <c r="B37" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C37" t="s">
-        <v>324</v>
-      </c>
-      <c r="D37" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F37" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>236</v>
       </c>
       <c r="B38" t="s">
-        <v>346</v>
+        <v>387</v>
       </c>
       <c r="C38" t="s">
-        <v>346</v>
+        <v>387</v>
       </c>
       <c r="D38" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+      <c r="E38" t="s">
+        <v>387</v>
+      </c>
+      <c r="F38" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>239</v>
       </c>
       <c r="B39" t="s">
+        <v>443</v>
+      </c>
+      <c r="C39" t="s">
         <v>280</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>281</v>
       </c>
-      <c r="D39" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E39" t="s">
+        <v>281</v>
+      </c>
+      <c r="F39" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>244</v>
       </c>
       <c r="B40" t="s">
-        <v>280</v>
+        <v>466</v>
       </c>
       <c r="C40" t="s">
-        <v>281</v>
-      </c>
-      <c r="D40" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+        <v>467</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F40" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>248</v>
       </c>
-      <c r="B41" t="s">
-        <v>328</v>
-      </c>
-      <c r="C41" t="s">
-        <v>329</v>
-      </c>
-      <c r="D41" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B41" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F41" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>250</v>
       </c>
       <c r="B42" t="s">
-        <v>346</v>
+        <v>387</v>
       </c>
       <c r="C42" t="s">
-        <v>346</v>
+        <v>387</v>
       </c>
       <c r="D42" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+      <c r="E42" t="s">
+        <v>387</v>
+      </c>
+      <c r="F42" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>253</v>
       </c>
       <c r="B43" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C43" t="s">
-        <v>324</v>
-      </c>
-      <c r="D43" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+        <v>319</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F43" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="B44" t="s">
-        <v>353</v>
-      </c>
-      <c r="C44" t="s">
-        <v>353</v>
-      </c>
-      <c r="D44" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B44" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>440</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>464</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>355</v>
+        <v>346</v>
       </c>
       <c r="B45" t="s">
-        <v>312</v>
+        <v>453</v>
       </c>
       <c r="C45" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="D45" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+        <v>311</v>
+      </c>
+      <c r="E45" t="s">
+        <v>462</v>
+      </c>
+      <c r="F45" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>258</v>
       </c>
       <c r="B46" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C46" t="s">
-        <v>324</v>
-      </c>
-      <c r="D46" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F46" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>262</v>
       </c>
       <c r="B47" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C47" t="s">
-        <v>324</v>
-      </c>
-      <c r="D47" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F47" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>359</v>
-      </c>
-      <c r="B48" t="s">
-        <v>328</v>
-      </c>
-      <c r="C48" t="s">
-        <v>329</v>
-      </c>
-      <c r="D48" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+        <v>350</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F48" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>264</v>
       </c>
       <c r="B49" t="s">
-        <v>296</v>
+        <v>447</v>
       </c>
       <c r="C49" t="s">
-        <v>316</v>
-      </c>
-      <c r="D49" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+        <v>295</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="F49" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="9" t="s">
         <v>268</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="E50" s="10" t="s">
+        <v>464</v>
+      </c>
+      <c r="F50" s="9" t="s">
         <v>353</v>
       </c>
-      <c r="C50" t="s">
-        <v>353</v>
-      </c>
-      <c r="D50" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>270</v>
       </c>
       <c r="B51" t="s">
-        <v>323</v>
+        <v>455</v>
       </c>
       <c r="C51" t="s">
-        <v>324</v>
-      </c>
-      <c r="D51" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F51" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>435</v>
+      </c>
+      <c r="B52" t="s">
         <v>446</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>288</v>
       </c>
-      <c r="C52" t="s">
-        <v>444</v>
-      </c>
-      <c r="D52" t="s">
-        <v>445</v>
+      <c r="D52" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="F52" t="s">
+        <v>434</v>
       </c>
     </row>
   </sheetData>
@@ -4328,87 +4736,87 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>364</v>
+        <v>355</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>365</v>
+        <v>356</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>369</v>
+        <v>360</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>374</v>
+        <v>365</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>375</v>
+        <v>366</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>376</v>
+        <v>367</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -4416,10 +4824,10 @@
         <v>122</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
@@ -4427,31 +4835,31 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -4474,18 +4882,18 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>385</v>
+        <v>376</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>386</v>
+        <v>377</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>279</v>
@@ -4493,52 +4901,52 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>28</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>394</v>
+        <v>385</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>28</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>399</v>
+        <v>390</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>28</v>
@@ -4547,24 +4955,24 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>28</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>401</v>
+        <v>392</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>28</v>
@@ -4587,23 +4995,23 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -4611,71 +5019,71 @@
         <v>145</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>414</v>
+        <v>405</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>415</v>
+        <v>406</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
       <c r="B11" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
       <c r="B12" t="s">
-        <v>422</v>
+        <v>413</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>423</v>
+        <v>414</v>
       </c>
       <c r="B13" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>
@@ -4695,64 +5103,64 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>425</v>
+        <v>416</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>426</v>
+        <v>417</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>427</v>
+        <v>418</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>429</v>
+        <v>420</v>
       </c>
       <c r="B4" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="C4" t="s">
-        <v>431</v>
+        <v>422</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>432</v>
+        <v>423</v>
       </c>
       <c r="B5" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="C5" t="s">
-        <v>431</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>433</v>
+        <v>424</v>
       </c>
       <c r="B6" t="s">
-        <v>434</v>
+        <v>425</v>
       </c>
       <c r="C6" t="s">
-        <v>435</v>
+        <v>426</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>436</v>
+        <v>427</v>
       </c>
       <c r="B7" t="s">
-        <v>434</v>
+        <v>425</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>437</v>
+        <v>428</v>
       </c>
       <c r="B8" t="s">
         <v>36</v>

</xml_diff>

<commit_message>
Output cleanup, three fixes, and dead-code removal
</commit_message>
<xml_diff>
--- a/config/kabelconfig.xlsx
+++ b/config/kabelconfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\io2cable\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197AF570-5A49-4F63-8B30-C6A0E4847FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1FB9B2C-A0EB-4D37-8A08-0F731146DFD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="77070" windowHeight="21150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0_Parameters" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="478">
   <si>
     <t>Step 0 — fill in per project BEFORE generation. Yellow fields are mandatory. Values in 'opties' (geen/erco/derden) are literal keys read by the engine — keep them as-is.</t>
   </si>
@@ -1328,9 +1328,6 @@
     <t>in technische ruimte</t>
   </si>
   <si>
-    <t>DRAK</t>
-  </si>
-  <si>
     <t>nsb8btn</t>
   </si>
   <si>
@@ -1443,6 +1440,39 @@
   </si>
   <si>
     <t>DRAK SIGK CCA 1X4X0,8 2501 MT</t>
+  </si>
+  <si>
+    <t>JOBA</t>
+  </si>
+  <si>
+    <t>resetknop</t>
+  </si>
+  <si>
+    <t>reset storingen</t>
+  </si>
+  <si>
+    <t>reset drukknop</t>
+  </si>
+  <si>
+    <t>installatie automaten</t>
+  </si>
+  <si>
+    <t>automaat 230V</t>
+  </si>
+  <si>
+    <t>automaat 24V</t>
+  </si>
+  <si>
+    <t>netwatcher</t>
+  </si>
+  <si>
+    <t>PANEL_INTERN</t>
+  </si>
+  <si>
+    <t>2195-06</t>
+  </si>
+  <si>
+    <t>7267</t>
   </si>
 </sst>
 </file>
@@ -1548,7 +1578,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1558,13 +1588,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1949,7 +1978,7 @@
         <v>17</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>18</v>
@@ -1963,7 +1992,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>429</v>
+        <v>467</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>21</v>
@@ -2075,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D122"/>
+  <dimension ref="A1:D129"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -3675,30 +3704,128 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B121" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C121">
         <v>70</v>
       </c>
       <c r="D121" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B122" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C122">
         <v>70</v>
       </c>
       <c r="D122" t="s">
-        <v>433</v>
+        <v>432</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>468</v>
+      </c>
+      <c r="B123" t="s">
+        <v>475</v>
+      </c>
+      <c r="C123">
+        <v>85</v>
+      </c>
+      <c r="D123">
+        <v>7267</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>469</v>
+      </c>
+      <c r="B124" t="s">
+        <v>475</v>
+      </c>
+      <c r="C124">
+        <v>85</v>
+      </c>
+      <c r="D124" s="9" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>470</v>
+      </c>
+      <c r="B125" t="s">
+        <v>475</v>
+      </c>
+      <c r="C125">
+        <v>85</v>
+      </c>
+      <c r="D125" s="9" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>471</v>
+      </c>
+      <c r="B126" t="s">
+        <v>475</v>
+      </c>
+      <c r="C126">
+        <v>85</v>
+      </c>
+      <c r="D126" s="9" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>472</v>
+      </c>
+      <c r="B127" t="s">
+        <v>475</v>
+      </c>
+      <c r="C127">
+        <v>85</v>
+      </c>
+      <c r="D127" s="9" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>473</v>
+      </c>
+      <c r="B128" t="s">
+        <v>475</v>
+      </c>
+      <c r="C128">
+        <v>85</v>
+      </c>
+      <c r="D128" s="9" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>474</v>
+      </c>
+      <c r="B129" t="s">
+        <v>475</v>
+      </c>
+      <c r="C129">
+        <v>85</v>
+      </c>
+      <c r="D129" s="9" t="s">
+        <v>476</v>
       </c>
     </row>
   </sheetData>
@@ -3726,7 +3853,7 @@
         <v>49</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>277</v>
@@ -3735,7 +3862,7 @@
         <v>278</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>279</v>
@@ -3746,7 +3873,7 @@
         <v>89</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>280</v>
@@ -3755,7 +3882,7 @@
         <v>281</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>282</v>
@@ -3766,7 +3893,7 @@
         <v>118</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>283</v>
@@ -3775,7 +3902,7 @@
         <v>281</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>284</v>
@@ -3786,7 +3913,7 @@
         <v>108</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>285</v>
@@ -3806,7 +3933,7 @@
         <v>287</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>283</v>
@@ -3815,7 +3942,7 @@
         <v>281</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F7" s="3"/>
     </row>
@@ -3824,7 +3951,7 @@
         <v>75</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>288</v>
@@ -3833,29 +3960,29 @@
         <v>289</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F8" s="3" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="9" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+    <row r="9" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>445</v>
-      </c>
-      <c r="C9" s="7" t="s">
+      <c r="B9" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>458</v>
-      </c>
-      <c r="F9" s="7" t="s">
+      <c r="E9" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>292</v>
       </c>
     </row>
@@ -3864,7 +3991,7 @@
         <v>98</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>285</v>
@@ -3873,7 +4000,7 @@
         <v>289</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F10" s="3"/>
     </row>
@@ -3882,7 +4009,7 @@
         <v>293</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>288</v>
@@ -3891,7 +4018,7 @@
         <v>289</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>294</v>
@@ -3902,7 +4029,7 @@
         <v>112</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>285</v>
@@ -3911,7 +4038,7 @@
         <v>289</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F12" s="3"/>
     </row>
@@ -3920,7 +4047,7 @@
         <v>94</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>295</v>
@@ -3929,7 +4056,7 @@
         <v>296</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>297</v>
@@ -3940,7 +4067,7 @@
         <v>101</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>298</v>
@@ -3949,7 +4076,7 @@
         <v>299</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>300</v>
@@ -3960,7 +4087,7 @@
         <v>103</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>285</v>
@@ -3969,7 +4096,7 @@
         <v>281</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>301</v>
@@ -3980,10 +4107,10 @@
         <v>114</v>
       </c>
       <c r="B16" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C16" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>302</v>
@@ -4000,7 +4127,7 @@
         <v>159</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>304</v>
@@ -4015,23 +4142,23 @@
         <v>305</v>
       </c>
     </row>
-    <row r="18" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="9" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>165</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>451</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>437</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>451</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>437</v>
-      </c>
-      <c r="F18" s="9" t="s">
+      <c r="B18" t="s">
+        <v>450</v>
+      </c>
+      <c r="C18" t="s">
+        <v>436</v>
+      </c>
+      <c r="D18" t="s">
+        <v>450</v>
+      </c>
+      <c r="E18" t="s">
+        <v>436</v>
+      </c>
+      <c r="F18" t="s">
         <v>306</v>
       </c>
     </row>
@@ -4040,7 +4167,7 @@
         <v>174</v>
       </c>
       <c r="B19" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C19" t="s">
         <v>307</v>
@@ -4049,7 +4176,7 @@
         <v>308</v>
       </c>
       <c r="E19" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="F19" t="s">
         <v>309</v>
@@ -4060,7 +4187,7 @@
         <v>181</v>
       </c>
       <c r="B20" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C20" t="s">
         <v>310</v>
@@ -4069,7 +4196,7 @@
         <v>311</v>
       </c>
       <c r="E20" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="F20" t="s">
         <v>312</v>
@@ -4080,7 +4207,7 @@
         <v>313</v>
       </c>
       <c r="B21" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C21" t="s">
         <v>295</v>
@@ -4089,7 +4216,7 @@
         <v>299</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F21" t="s">
         <v>314</v>
@@ -4100,7 +4227,7 @@
         <v>185</v>
       </c>
       <c r="B22" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C22" t="s">
         <v>315</v>
@@ -4109,7 +4236,7 @@
         <v>316</v>
       </c>
       <c r="E22" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F22" t="s">
         <v>317</v>
@@ -4120,7 +4247,7 @@
         <v>188</v>
       </c>
       <c r="B23" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C23" t="s">
         <v>304</v>
@@ -4140,7 +4267,7 @@
         <v>192</v>
       </c>
       <c r="B24" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C24" t="s">
         <v>319</v>
@@ -4149,7 +4276,7 @@
         <v>289</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F24" t="s">
         <v>320</v>
@@ -4160,7 +4287,7 @@
         <v>195</v>
       </c>
       <c r="B25" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C25" t="s">
         <v>319</v>
@@ -4169,7 +4296,7 @@
         <v>289</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F25" t="s">
         <v>321</v>
@@ -4180,7 +4307,7 @@
         <v>198</v>
       </c>
       <c r="B26" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C26" t="s">
         <v>319</v>
@@ -4189,7 +4316,7 @@
         <v>289</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F26" t="s">
         <v>322</v>
@@ -4200,7 +4327,7 @@
         <v>201</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>288</v>
@@ -4220,7 +4347,7 @@
         <v>203</v>
       </c>
       <c r="B28" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C28" t="s">
         <v>319</v>
@@ -4229,7 +4356,7 @@
         <v>289</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F28" t="s">
         <v>324</v>
@@ -4240,7 +4367,7 @@
         <v>208</v>
       </c>
       <c r="B29" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C29" t="s">
         <v>319</v>
@@ -4249,7 +4376,7 @@
         <v>289</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F29" t="s">
         <v>325</v>
@@ -4280,7 +4407,7 @@
         <v>216</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>288</v>
@@ -4289,7 +4416,7 @@
         <v>289</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F31" t="s">
         <v>329</v>
@@ -4320,7 +4447,7 @@
         <v>222</v>
       </c>
       <c r="B33" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C33" t="s">
         <v>319</v>
@@ -4329,7 +4456,7 @@
         <v>289</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F33" t="s">
         <v>333</v>
@@ -4340,7 +4467,7 @@
         <v>225</v>
       </c>
       <c r="B34" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C34" t="s">
         <v>319</v>
@@ -4349,7 +4476,7 @@
         <v>289</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F34" t="s">
         <v>334</v>
@@ -4360,16 +4487,16 @@
         <v>229</v>
       </c>
       <c r="B35" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C35" t="s">
         <v>295</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="F35" t="s">
         <v>335</v>
@@ -4380,7 +4507,7 @@
         <v>232</v>
       </c>
       <c r="B36" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C36" t="s">
         <v>319</v>
@@ -4400,7 +4527,7 @@
         <v>234</v>
       </c>
       <c r="B37" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C37" t="s">
         <v>319</v>
@@ -4409,7 +4536,7 @@
         <v>289</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F37" t="s">
         <v>337</v>
@@ -4440,7 +4567,7 @@
         <v>239</v>
       </c>
       <c r="B39" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C39" t="s">
         <v>280</v>
@@ -4460,10 +4587,10 @@
         <v>244</v>
       </c>
       <c r="B40" t="s">
+        <v>465</v>
+      </c>
+      <c r="C40" t="s">
         <v>466</v>
-      </c>
-      <c r="C40" t="s">
-        <v>467</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>289</v>
@@ -4480,7 +4607,7 @@
         <v>248</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>288</v>
@@ -4489,7 +4616,7 @@
         <v>289</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F41" t="s">
         <v>342</v>
@@ -4520,7 +4647,7 @@
         <v>253</v>
       </c>
       <c r="B43" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C43" t="s">
         <v>319</v>
@@ -4529,33 +4656,33 @@
         <v>289</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F43" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="44" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="9" t="s">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>255</v>
       </c>
-      <c r="B44" s="10" t="s">
+      <c r="B44" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="C44" s="10" t="s">
-        <v>440</v>
-      </c>
-      <c r="D44" s="10" t="s">
+      <c r="C44" s="8" t="s">
+        <v>439</v>
+      </c>
+      <c r="D44" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="E44" s="10" t="s">
-        <v>464</v>
-      </c>
-      <c r="F44" s="9" t="s">
+      <c r="E44" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="F44" t="s">
         <v>345</v>
       </c>
-      <c r="G44" s="9" t="s">
-        <v>439</v>
+      <c r="G44" t="s">
+        <v>438</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -4563,7 +4690,7 @@
         <v>346</v>
       </c>
       <c r="B45" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C45" t="s">
         <v>310</v>
@@ -4572,7 +4699,7 @@
         <v>311</v>
       </c>
       <c r="E45" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="F45" t="s">
         <v>347</v>
@@ -4583,7 +4710,7 @@
         <v>258</v>
       </c>
       <c r="B46" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C46" t="s">
         <v>319</v>
@@ -4592,7 +4719,7 @@
         <v>289</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F46" t="s">
         <v>348</v>
@@ -4603,7 +4730,7 @@
         <v>262</v>
       </c>
       <c r="B47" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C47" t="s">
         <v>319</v>
@@ -4612,7 +4739,7 @@
         <v>289</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F47" t="s">
         <v>349</v>
@@ -4623,7 +4750,7 @@
         <v>350</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>288</v>
@@ -4643,7 +4770,7 @@
         <v>264</v>
       </c>
       <c r="B49" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C49" t="s">
         <v>295</v>
@@ -4652,29 +4779,29 @@
         <v>299</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F49" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="50" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="9" t="s">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>268</v>
       </c>
-      <c r="B50" s="10" t="s">
+      <c r="B50" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="D50" s="10" t="s">
+      <c r="D50" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="E50" s="10" t="s">
-        <v>464</v>
-      </c>
-      <c r="F50" s="9" t="s">
+      <c r="E50" s="8" t="s">
+        <v>463</v>
+      </c>
+      <c r="F50" t="s">
         <v>353</v>
       </c>
     </row>
@@ -4683,7 +4810,7 @@
         <v>270</v>
       </c>
       <c r="B51" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C51" t="s">
         <v>319</v>
@@ -4700,10 +4827,10 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B52" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C52" t="s">
         <v>288</v>
@@ -4712,10 +4839,10 @@
         <v>289</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F52" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
classify: procescode in match text + DO fallback to KLEP_OD_ZONDER_TERUGMELDING
</commit_message>
<xml_diff>
--- a/config/kabelconfig.xlsx
+++ b/config/kabelconfig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\io2cable\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1FB9B2C-A0EB-4D37-8A08-0F731146DFD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EB6A391-5ABB-4ACA-97B2-83C979100CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="491">
   <si>
     <t>Step 0 — fill in per project BEFORE generation. Yellow fields are mandatory. Values in 'opties' (geen/erco/derden) are literal keys read by the engine — keep them as-is.</t>
   </si>
@@ -1442,9 +1442,6 @@
     <t>DRAK SIGK CCA 1X4X0,8 2501 MT</t>
   </si>
   <si>
-    <t>JOBA</t>
-  </si>
-  <si>
     <t>resetknop</t>
   </si>
   <si>
@@ -1473,6 +1470,48 @@
   </si>
   <si>
     <t>7267</t>
+  </si>
+  <si>
+    <t>afsluiter</t>
+  </si>
+  <si>
+    <t>kogelafsluiter</t>
+  </si>
+  <si>
+    <t>busafsluitmodule</t>
+  </si>
+  <si>
+    <t>netwerkmodule</t>
+  </si>
+  <si>
+    <t>communicatiebase</t>
+  </si>
+  <si>
+    <t>basismodule</t>
+  </si>
+  <si>
+    <t>aqb2005</t>
+  </si>
+  <si>
+    <t>aqb2002</t>
+  </si>
+  <si>
+    <t>connection set</t>
+  </si>
+  <si>
+    <t>ingangsbase</t>
+  </si>
+  <si>
+    <t>uitgangsbase</t>
+  </si>
+  <si>
+    <t>priva blue id</t>
+  </si>
+  <si>
+    <t>DRAK</t>
+  </si>
+  <si>
+    <t>KLEP_OD_ZONDER_TERUGMELDING</t>
   </si>
 </sst>
 </file>
@@ -1532,7 +1571,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1547,6 +1586,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1578,7 +1623,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1594,6 +1639,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1992,7 +2038,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>467</v>
+        <v>489</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>21</v>
@@ -2104,7 +2150,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D129"/>
+  <dimension ref="A1:D141"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -3732,10 +3778,10 @@
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B123" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C123">
         <v>85</v>
@@ -3746,86 +3792,254 @@
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="B124" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C124">
         <v>85</v>
       </c>
       <c r="D124" s="9" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B125" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C125">
         <v>85</v>
       </c>
       <c r="D125" s="9" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B126" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C126">
         <v>85</v>
       </c>
       <c r="D126" s="9" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B127" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C127">
         <v>85</v>
       </c>
       <c r="D127" s="9" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B128" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C128">
         <v>85</v>
       </c>
       <c r="D128" s="9" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
+        <v>473</v>
+      </c>
+      <c r="B129" t="s">
         <v>474</v>
-      </c>
-      <c r="B129" t="s">
-        <v>475</v>
       </c>
       <c r="C129">
         <v>85</v>
       </c>
       <c r="D129" s="9" t="s">
-        <v>476</v>
+        <v>475</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>477</v>
+      </c>
+      <c r="B130" t="s">
+        <v>101</v>
+      </c>
+      <c r="C130">
+        <v>20</v>
+      </c>
+      <c r="D130">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>478</v>
+      </c>
+      <c r="B131" t="s">
+        <v>101</v>
+      </c>
+      <c r="C131">
+        <v>40</v>
+      </c>
+      <c r="D131">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>488</v>
+      </c>
+      <c r="B132" t="s">
+        <v>474</v>
+      </c>
+      <c r="C132">
+        <v>85</v>
+      </c>
+      <c r="D132">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>479</v>
+      </c>
+      <c r="B133" t="s">
+        <v>474</v>
+      </c>
+      <c r="C133">
+        <v>85</v>
+      </c>
+      <c r="D133">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>480</v>
+      </c>
+      <c r="B134" t="s">
+        <v>474</v>
+      </c>
+      <c r="C134">
+        <v>85</v>
+      </c>
+      <c r="D134">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>481</v>
+      </c>
+      <c r="B135" t="s">
+        <v>474</v>
+      </c>
+      <c r="C135">
+        <v>85</v>
+      </c>
+      <c r="D135">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>486</v>
+      </c>
+      <c r="B136" t="s">
+        <v>474</v>
+      </c>
+      <c r="C136">
+        <v>85</v>
+      </c>
+      <c r="D136">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>487</v>
+      </c>
+      <c r="B137" t="s">
+        <v>474</v>
+      </c>
+      <c r="C137">
+        <v>85</v>
+      </c>
+      <c r="D137">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>482</v>
+      </c>
+      <c r="B138" t="s">
+        <v>474</v>
+      </c>
+      <c r="C138">
+        <v>85</v>
+      </c>
+      <c r="D138">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>483</v>
+      </c>
+      <c r="B139" t="s">
+        <v>79</v>
+      </c>
+      <c r="C139">
+        <v>90</v>
+      </c>
+      <c r="D139">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>484</v>
+      </c>
+      <c r="B140" t="s">
+        <v>79</v>
+      </c>
+      <c r="C140">
+        <v>90</v>
+      </c>
+      <c r="D140">
+        <v>7222</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>485</v>
+      </c>
+      <c r="B141" t="s">
+        <v>79</v>
+      </c>
+      <c r="C141">
+        <v>90</v>
+      </c>
+      <c r="D141">
+        <v>7222</v>
       </c>
     </row>
   </sheetData>
@@ -3835,7 +4049,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -4843,6 +5057,17 @@
       </c>
       <c r="F52" t="s">
         <v>433</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="10" t="s">
+        <v>490</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>454</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>319</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made BRANDVENTILATIESCHAKEL afvoer and toevoer merge in output
</commit_message>
<xml_diff>
--- a/config/kabelconfig.xlsx
+++ b/config/kabelconfig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\io2cable\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CB53452-426E-4F5E-9930-7FD464BA5A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D9AB56-E9A5-4934-991B-7DF923725180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="492">
   <si>
     <t>Step 2 — classification dictionary. The longest / highest-priority match wins. Add every manual correction here (the system gets smarter with each project). The 'functietype' codes are keys shared with tab 2_Kabelkeuze — keep them identical.</t>
   </si>
@@ -1496,6 +1496,12 @@
   </si>
   <si>
     <t>MBUS</t>
+  </si>
+  <si>
+    <t>brandschakelaar toevoer</t>
+  </si>
+  <si>
+    <t>brandschakelaar afvoer</t>
   </si>
 </sst>
 </file>
@@ -2134,7 +2140,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D141"/>
+  <dimension ref="A1:D143"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -4024,6 +4030,34 @@
       </c>
       <c r="D141">
         <v>7222</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>490</v>
+      </c>
+      <c r="B142" t="s">
+        <v>182</v>
+      </c>
+      <c r="C142">
+        <v>75</v>
+      </c>
+      <c r="D142">
+        <v>7224</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>491</v>
+      </c>
+      <c r="B143" t="s">
+        <v>182</v>
+      </c>
+      <c r="C143">
+        <v>75</v>
+      </c>
+      <c r="D143">
+        <v>7224</v>
       </c>
     </row>
   </sheetData>
@@ -4685,10 +4719,10 @@
         <v>182</v>
       </c>
       <c r="B35" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="C35" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>381</v>

</xml_diff>

<commit_message>
added regelafsluiter open/ditch and improved mod titles plus updated change and questions log at the end of the day
</commit_message>
<xml_diff>
--- a/config/kabelconfig.xlsx
+++ b/config/kabelconfig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\io2cable\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D9AB56-E9A5-4934-991B-7DF923725180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF0CC26-B6A2-4BF7-8980-0F31DF2EF53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="494">
   <si>
     <t>Step 2 — classification dictionary. The longest / highest-priority match wins. Add every manual correction here (the system gets smarter with each project). The 'functietype' codes are keys shared with tab 2_Kabelkeuze — keep them identical.</t>
   </si>
@@ -1502,6 +1502,12 @@
   </si>
   <si>
     <t>brandschakelaar afvoer</t>
+  </si>
+  <si>
+    <t>JOBA ST.STR B2CA HCHOZ 5X1 MT</t>
+  </si>
+  <si>
+    <t>JOBA ST.STR CCA HCHOZ 5X1 MT</t>
   </si>
 </sst>
 </file>
@@ -4305,10 +4311,10 @@
         <v>337</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>338</v>
+        <v>381</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>339</v>
+        <v>382</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>340</v>
@@ -4325,10 +4331,10 @@
         <v>319</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>312</v>
+        <v>492</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>313</v>
+        <v>493</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>341</v>
@@ -4848,7 +4854,7 @@
         <v>324</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F41" t="s">
         <v>392</v>
@@ -5042,10 +5048,10 @@
         <v>223</v>
       </c>
       <c r="B51" t="s">
-        <v>366</v>
+        <v>322</v>
       </c>
       <c r="C51" t="s">
-        <v>367</v>
+        <v>323</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>324</v>
@@ -5071,7 +5077,7 @@
         <v>324</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F52" t="s">
         <v>409</v>

</xml_diff>

<commit_message>
addded the grouping in the output back
</commit_message>
<xml_diff>
--- a/config/kabelconfig.xlsx
+++ b/config/kabelconfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\io2cable\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB738041-3A18-47BC-B0D5-15DBFB97452A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9C1FE19-2FFC-47A6-92D6-46B0C10DACD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0_Parameters" sheetId="1" r:id="rId1"/>
@@ -859,9 +859,6 @@
     <t>signaalfamilie</t>
   </si>
   <si>
-    <t>DRAK</t>
-  </si>
-  <si>
     <t>DRAK / JOBA</t>
   </si>
   <si>
@@ -1529,6 +1526,9 @@
   </si>
   <si>
     <t>VAV_SIGNAAL</t>
+  </si>
+  <si>
+    <t>JOBA</t>
   </si>
 </sst>
 </file>
@@ -2047,7 +2047,7 @@
         <v>273</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>274</v>
@@ -2061,109 +2061,109 @@
         <v>276</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>278</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>282</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>286</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>290</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>292</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>293</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
+        <v>294</v>
+      </c>
+      <c r="B14" t="s">
         <v>295</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>296</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>297</v>
-      </c>
-      <c r="D14" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
+        <v>298</v>
+      </c>
+      <c r="B15" t="s">
+        <v>295</v>
+      </c>
+      <c r="C15" t="s">
+        <v>296</v>
+      </c>
+      <c r="D15" t="s">
         <v>299</v>
-      </c>
-      <c r="B15" t="s">
-        <v>296</v>
-      </c>
-      <c r="C15" t="s">
-        <v>297</v>
-      </c>
-      <c r="D15" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
+        <v>300</v>
+      </c>
+      <c r="B16" t="s">
         <v>301</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>296</v>
+      </c>
+      <c r="D16" t="s">
         <v>302</v>
-      </c>
-      <c r="C16" t="s">
-        <v>297</v>
-      </c>
-      <c r="D16" t="s">
-        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -2506,7 +2506,7 @@
         <v>49</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C27" s="3">
         <v>80</v>
@@ -4067,7 +4067,7 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="B142" t="s">
         <v>182</v>
@@ -4081,7 +4081,7 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="B143" t="s">
         <v>182</v>
@@ -4095,10 +4095,10 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B144" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C144">
         <v>75</v>
@@ -4109,10 +4109,10 @@
     </row>
     <row r="145" spans="1:4">
       <c r="A145" t="s">
+        <v>498</v>
+      </c>
+      <c r="B145" s="11" t="s">
         <v>499</v>
-      </c>
-      <c r="B145" s="11" t="s">
-        <v>500</v>
       </c>
       <c r="C145">
         <v>45</v>
@@ -4138,7 +4138,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -4146,19 +4146,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>308</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -4166,19 +4166,19 @@
         <v>42</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>311</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>313</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -4186,19 +4186,19 @@
         <v>71</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>316</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -4206,36 +4206,36 @@
         <v>61</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>319</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>315</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>316</v>
-      </c>
       <c r="D7" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>312</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>313</v>
       </c>
       <c r="F7" s="3"/>
     </row>
@@ -4244,39 +4244,39 @@
         <v>28</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>325</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="7" customFormat="1">
       <c r="A9" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>327</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -4284,37 +4284,37 @@
         <v>51</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>319</v>
-      </c>
       <c r="D10" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>324</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>325</v>
       </c>
       <c r="F10" s="3"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>329</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -4322,16 +4322,16 @@
         <v>65</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>319</v>
-      </c>
       <c r="D12" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>324</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>325</v>
       </c>
       <c r="F12" s="3"/>
     </row>
@@ -4340,19 +4340,19 @@
         <v>47</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>334</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -4360,19 +4360,19 @@
         <v>54</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>337</v>
-      </c>
       <c r="D14" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>382</v>
-      </c>
       <c r="F14" s="3" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -4380,19 +4380,19 @@
         <v>56</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>319</v>
-      </c>
       <c r="D15" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>491</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>492</v>
-      </c>
       <c r="F15" s="3" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -4400,19 +4400,19 @@
         <v>67</v>
       </c>
       <c r="B16" t="s">
+        <v>341</v>
+      </c>
+      <c r="C16" t="s">
         <v>342</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>344</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -4420,19 +4420,19 @@
         <v>112</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>347</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>338</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>338</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -4440,19 +4440,19 @@
         <v>118</v>
       </c>
       <c r="B18" t="s">
+        <v>348</v>
+      </c>
+      <c r="C18" t="s">
         <v>349</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
+        <v>348</v>
+      </c>
+      <c r="E18" t="s">
+        <v>349</v>
+      </c>
+      <c r="F18" t="s">
         <v>350</v>
-      </c>
-      <c r="D18" t="s">
-        <v>349</v>
-      </c>
-      <c r="E18" t="s">
-        <v>350</v>
-      </c>
-      <c r="F18" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -4460,19 +4460,19 @@
         <v>127</v>
       </c>
       <c r="B19" t="s">
+        <v>351</v>
+      </c>
+      <c r="C19" t="s">
         <v>352</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>353</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>354</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>355</v>
-      </c>
-      <c r="F19" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -4480,39 +4480,39 @@
         <v>134</v>
       </c>
       <c r="B20" t="s">
+        <v>356</v>
+      </c>
+      <c r="C20" t="s">
         <v>357</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>358</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E20" t="s">
         <v>359</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>360</v>
-      </c>
-      <c r="F20" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
+        <v>361</v>
+      </c>
+      <c r="B21" t="s">
+        <v>330</v>
+      </c>
+      <c r="C21" t="s">
+        <v>331</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="F21" t="s">
         <v>362</v>
-      </c>
-      <c r="B21" t="s">
-        <v>331</v>
-      </c>
-      <c r="C21" t="s">
-        <v>332</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>338</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>339</v>
-      </c>
-      <c r="F21" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -4520,19 +4520,19 @@
         <v>138</v>
       </c>
       <c r="B22" t="s">
+        <v>351</v>
+      </c>
+      <c r="C22" t="s">
         <v>352</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>353</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>354</v>
       </c>
-      <c r="E22" t="s">
-        <v>355</v>
-      </c>
       <c r="F22" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -4540,19 +4540,19 @@
         <v>141</v>
       </c>
       <c r="B23" t="s">
+        <v>345</v>
+      </c>
+      <c r="C23" t="s">
         <v>346</v>
       </c>
-      <c r="C23" t="s">
-        <v>347</v>
-      </c>
       <c r="D23" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F23" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -4560,19 +4560,19 @@
         <v>145</v>
       </c>
       <c r="B24" t="s">
+        <v>365</v>
+      </c>
+      <c r="C24" t="s">
         <v>366</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="F24" t="s">
         <v>367</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="F24" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -4580,19 +4580,19 @@
         <v>148</v>
       </c>
       <c r="B25" t="s">
+        <v>365</v>
+      </c>
+      <c r="C25" t="s">
         <v>366</v>
       </c>
-      <c r="C25" t="s">
-        <v>367</v>
-      </c>
       <c r="D25" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E25" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F25" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -4600,19 +4600,19 @@
         <v>151</v>
       </c>
       <c r="B26" t="s">
+        <v>365</v>
+      </c>
+      <c r="C26" t="s">
         <v>366</v>
       </c>
-      <c r="C26" t="s">
-        <v>367</v>
-      </c>
       <c r="D26" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F26" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -4620,19 +4620,19 @@
         <v>154</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="D27" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>324</v>
-      </c>
       <c r="E27" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F27" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -4640,19 +4640,19 @@
         <v>156</v>
       </c>
       <c r="B28" t="s">
+        <v>365</v>
+      </c>
+      <c r="C28" t="s">
         <v>366</v>
       </c>
-      <c r="C28" t="s">
-        <v>367</v>
-      </c>
       <c r="D28" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E28" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F28" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -4660,19 +4660,19 @@
         <v>161</v>
       </c>
       <c r="B29" t="s">
+        <v>365</v>
+      </c>
+      <c r="C29" t="s">
         <v>366</v>
       </c>
-      <c r="C29" t="s">
-        <v>367</v>
-      </c>
       <c r="D29" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E29" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F29" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -4680,19 +4680,19 @@
         <v>164</v>
       </c>
       <c r="B30" t="s">
+        <v>373</v>
+      </c>
+      <c r="C30" t="s">
         <v>374</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
+        <v>373</v>
+      </c>
+      <c r="E30" t="s">
+        <v>374</v>
+      </c>
+      <c r="F30" t="s">
         <v>375</v>
-      </c>
-      <c r="D30" t="s">
-        <v>374</v>
-      </c>
-      <c r="E30" t="s">
-        <v>375</v>
-      </c>
-      <c r="F30" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -4700,19 +4700,19 @@
         <v>169</v>
       </c>
       <c r="B31" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="D31" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="E31" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E31" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F31" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -4720,19 +4720,19 @@
         <v>172</v>
       </c>
       <c r="B32" t="s">
+        <v>358</v>
+      </c>
+      <c r="C32" t="s">
         <v>359</v>
       </c>
-      <c r="C32" t="s">
-        <v>360</v>
-      </c>
       <c r="D32" t="s">
+        <v>358</v>
+      </c>
+      <c r="E32" t="s">
         <v>359</v>
       </c>
-      <c r="E32" t="s">
-        <v>360</v>
-      </c>
       <c r="F32" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -4740,19 +4740,19 @@
         <v>175</v>
       </c>
       <c r="B33" t="s">
+        <v>365</v>
+      </c>
+      <c r="C33" t="s">
         <v>366</v>
       </c>
-      <c r="C33" t="s">
-        <v>367</v>
-      </c>
       <c r="D33" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E33" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F33" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -4760,19 +4760,19 @@
         <v>178</v>
       </c>
       <c r="B34" t="s">
+        <v>365</v>
+      </c>
+      <c r="C34" t="s">
         <v>366</v>
       </c>
-      <c r="C34" t="s">
-        <v>367</v>
-      </c>
       <c r="D34" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E34" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F34" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -4780,19 +4780,19 @@
         <v>182</v>
       </c>
       <c r="B35" t="s">
+        <v>335</v>
+      </c>
+      <c r="C35" t="s">
         <v>336</v>
       </c>
-      <c r="C35" t="s">
-        <v>337</v>
-      </c>
       <c r="D35" s="3" t="s">
+        <v>380</v>
+      </c>
+      <c r="E35" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="F35" t="s">
         <v>382</v>
-      </c>
-      <c r="F35" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -4800,19 +4800,19 @@
         <v>185</v>
       </c>
       <c r="B36" t="s">
+        <v>322</v>
+      </c>
+      <c r="C36" t="s">
+        <v>322</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="C36" t="s">
+      <c r="E36" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="D36" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>324</v>
-      </c>
       <c r="F36" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -4820,19 +4820,19 @@
         <v>187</v>
       </c>
       <c r="B37" t="s">
+        <v>365</v>
+      </c>
+      <c r="C37" t="s">
         <v>366</v>
       </c>
-      <c r="C37" t="s">
-        <v>367</v>
-      </c>
       <c r="D37" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E37" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E37" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F37" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -4840,19 +4840,19 @@
         <v>189</v>
       </c>
       <c r="B38" t="s">
+        <v>385</v>
+      </c>
+      <c r="C38" t="s">
+        <v>385</v>
+      </c>
+      <c r="D38" t="s">
+        <v>385</v>
+      </c>
+      <c r="E38" t="s">
+        <v>385</v>
+      </c>
+      <c r="F38" t="s">
         <v>386</v>
-      </c>
-      <c r="C38" t="s">
-        <v>386</v>
-      </c>
-      <c r="D38" t="s">
-        <v>386</v>
-      </c>
-      <c r="E38" t="s">
-        <v>386</v>
-      </c>
-      <c r="F38" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -4860,19 +4860,19 @@
         <v>192</v>
       </c>
       <c r="B39" t="s">
+        <v>309</v>
+      </c>
+      <c r="C39" t="s">
         <v>310</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>311</v>
       </c>
-      <c r="D39" t="s">
-        <v>312</v>
-      </c>
       <c r="E39" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F39" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -4880,19 +4880,19 @@
         <v>197</v>
       </c>
       <c r="B40" t="s">
+        <v>388</v>
+      </c>
+      <c r="C40" t="s">
         <v>389</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="F40" t="s">
         <v>390</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="F40" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -4900,19 +4900,19 @@
         <v>201</v>
       </c>
       <c r="B41" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="D41" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="D41" s="3" t="s">
-        <v>324</v>
-      </c>
       <c r="E41" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F41" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -4920,19 +4920,19 @@
         <v>203</v>
       </c>
       <c r="B42" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C42" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D42" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E42" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F42" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -4940,19 +4940,19 @@
         <v>206</v>
       </c>
       <c r="B43" t="s">
+        <v>365</v>
+      </c>
+      <c r="C43" t="s">
         <v>366</v>
       </c>
-      <c r="C43" t="s">
-        <v>367</v>
-      </c>
       <c r="D43" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F43" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -4960,42 +4960,42 @@
         <v>208</v>
       </c>
       <c r="B44" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="C44" s="8" t="s">
         <v>395</v>
       </c>
-      <c r="C44" s="8" t="s">
+      <c r="D44" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="E44" s="8" t="s">
         <v>396</v>
       </c>
-      <c r="D44" s="8" t="s">
-        <v>395</v>
-      </c>
-      <c r="E44" s="8" t="s">
+      <c r="F44" t="s">
         <v>397</v>
       </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
         <v>398</v>
-      </c>
-      <c r="G44" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" t="s">
+        <v>399</v>
+      </c>
+      <c r="B45" t="s">
+        <v>356</v>
+      </c>
+      <c r="C45" t="s">
+        <v>357</v>
+      </c>
+      <c r="D45" t="s">
+        <v>358</v>
+      </c>
+      <c r="E45" t="s">
+        <v>359</v>
+      </c>
+      <c r="F45" t="s">
         <v>400</v>
-      </c>
-      <c r="B45" t="s">
-        <v>357</v>
-      </c>
-      <c r="C45" t="s">
-        <v>358</v>
-      </c>
-      <c r="D45" t="s">
-        <v>359</v>
-      </c>
-      <c r="E45" t="s">
-        <v>360</v>
-      </c>
-      <c r="F45" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -5003,19 +5003,19 @@
         <v>211</v>
       </c>
       <c r="B46" t="s">
+        <v>365</v>
+      </c>
+      <c r="C46" t="s">
         <v>366</v>
       </c>
-      <c r="C46" t="s">
-        <v>367</v>
-      </c>
       <c r="D46" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E46" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E46" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F46" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -5023,39 +5023,39 @@
         <v>215</v>
       </c>
       <c r="B47" t="s">
+        <v>365</v>
+      </c>
+      <c r="C47" t="s">
         <v>366</v>
       </c>
-      <c r="C47" t="s">
-        <v>367</v>
-      </c>
       <c r="D47" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E47" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="E47" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="F47" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" t="s">
+        <v>403</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="F48" t="s">
         <v>404</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="F48" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -5063,19 +5063,19 @@
         <v>217</v>
       </c>
       <c r="B49" t="s">
+        <v>330</v>
+      </c>
+      <c r="C49" t="s">
         <v>331</v>
       </c>
-      <c r="C49" t="s">
-        <v>332</v>
-      </c>
       <c r="D49" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="E49" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="E49" s="3" t="s">
-        <v>339</v>
-      </c>
       <c r="F49" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -5083,19 +5083,19 @@
         <v>221</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F50" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -5103,19 +5103,19 @@
         <v>223</v>
       </c>
       <c r="B51" t="s">
+        <v>321</v>
+      </c>
+      <c r="C51" t="s">
         <v>322</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="D51" s="3" t="s">
-        <v>324</v>
-      </c>
       <c r="E51" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F51" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -5123,121 +5123,121 @@
         <v>230</v>
       </c>
       <c r="B52" t="s">
+        <v>321</v>
+      </c>
+      <c r="C52" t="s">
         <v>322</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="D52" s="3" t="s">
-        <v>324</v>
-      </c>
       <c r="E52" s="3" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F52" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="53" spans="1:6" s="10" customFormat="1">
       <c r="A53" s="10" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B53" s="10" t="s">
+        <v>365</v>
+      </c>
+      <c r="C53" s="10" t="s">
         <v>366</v>
-      </c>
-      <c r="C53" s="10" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="10" t="s">
+        <v>410</v>
+      </c>
+      <c r="B54" s="10" t="s">
         <v>411</v>
       </c>
-      <c r="B54" s="10" t="s">
+      <c r="C54" s="10" t="s">
+        <v>411</v>
+      </c>
+      <c r="D54" t="s">
+        <v>411</v>
+      </c>
+      <c r="E54" t="s">
+        <v>411</v>
+      </c>
+      <c r="F54" t="s">
         <v>412</v>
-      </c>
-      <c r="C54" s="10" t="s">
-        <v>412</v>
-      </c>
-      <c r="D54" t="s">
-        <v>412</v>
-      </c>
-      <c r="E54" t="s">
-        <v>412</v>
-      </c>
-      <c r="F54" t="s">
-        <v>413</v>
       </c>
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="B55" s="10" t="s">
         <v>414</v>
       </c>
-      <c r="B55" s="10" t="s">
+      <c r="C55" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="D55" t="s">
+        <v>414</v>
+      </c>
+      <c r="E55" t="s">
+        <v>414</v>
+      </c>
+      <c r="F55" t="s">
         <v>415</v>
-      </c>
-      <c r="C55" s="10" t="s">
-        <v>415</v>
-      </c>
-      <c r="D55" t="s">
-        <v>415</v>
-      </c>
-      <c r="E55" t="s">
-        <v>415</v>
-      </c>
-      <c r="F55" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="10" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B56" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="C56" s="10" t="s">
         <v>336</v>
       </c>
-      <c r="C56" s="10" t="s">
-        <v>337</v>
-      </c>
       <c r="D56" s="10" t="s">
+        <v>380</v>
+      </c>
+      <c r="E56" s="10" t="s">
         <v>381</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="10" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="B57" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C57" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="D57" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E57" s="3" t="s">
         <v>324</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="11" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B58" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C58" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="D58" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E58" s="3" t="s">
         <v>324</v>
-      </c>
-      <c r="E58" s="3" t="s">
-        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -5258,87 +5258,87 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="5" t="s">
         <v>422</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>423</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>424</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>425</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>353</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>354</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>429</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>430</v>
-      </c>
       <c r="C5" s="3" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="3" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -5346,10 +5346,10 @@
         <v>75</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
@@ -5357,31 +5357,31 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>434</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>435</v>
-      </c>
       <c r="C8" s="3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>436</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>437</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -5404,100 +5404,100 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>441</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>442</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>443</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
+        <v>444</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>445</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>447</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="3" t="s">
+        <v>448</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>449</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>450</v>
-      </c>
       <c r="C7" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>452</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="B9" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D9" s="3"/>
     </row>
@@ -5517,23 +5517,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>455</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>457</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>458</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -5541,71 +5541,71 @@
         <v>98</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>459</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>461</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>463</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>464</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>465</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>467</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
+        <v>468</v>
+      </c>
+      <c r="B11" t="s">
         <v>469</v>
-      </c>
-      <c r="B11" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
+        <v>470</v>
+      </c>
+      <c r="B12" t="s">
         <v>471</v>
-      </c>
-      <c r="B12" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
+        <v>472</v>
+      </c>
+      <c r="B13" t="s">
         <v>473</v>
-      </c>
-      <c r="B13" t="s">
-        <v>474</v>
       </c>
     </row>
   </sheetData>
@@ -5625,67 +5625,67 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="6" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>476</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>477</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>478</v>
+      </c>
+      <c r="B4" t="s">
         <v>479</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>480</v>
-      </c>
-      <c r="C4" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B5" t="s">
+        <v>479</v>
+      </c>
+      <c r="C5" t="s">
         <v>480</v>
-      </c>
-      <c r="C5" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
+        <v>482</v>
+      </c>
+      <c r="B6" t="s">
         <v>483</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>484</v>
-      </c>
-      <c r="C6" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B7" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
interpret - as none
</commit_message>
<xml_diff>
--- a/config/kabelconfig.xlsx
+++ b/config/kabelconfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\io2cable\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{582D07A1-7067-45D8-BD54-74E26D753A71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{585410AA-F8C1-4B0E-B531-332E76D82E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0_Parameters" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="510">
   <si>
     <t>Step 2 — classification dictionary. The longest / highest-priority match wins. Add every manual correction here (the system gets smarter with each project). The 'functietype' codes are keys shared with tab 2_Kabelkeuze — keep them identical.</t>
   </si>
@@ -1249,18 +1249,12 @@
     <t>KLEP_OD_ZONDER_TERUGMELDING</t>
   </si>
   <si>
-    <t>1x4x0,8</t>
-  </si>
-  <si>
     <t>pomp met 2 signalen (vrijgave/storing). Rick 2026-08-18 + CCA dictionary. Dictionary value is family-agnostic, so identical in all four columns. Pump-specific: dict gives a 3-signal KETEL 1x4x0,8 and a 2-signal VENTILATOR 2x2x0,8, so do NOT generalise the count rule.</t>
   </si>
   <si>
     <t>POMP_3_SIGNALEN</t>
   </si>
   <si>
-    <t>3x2x0,8</t>
-  </si>
-  <si>
     <t>pomp met 3 signalen (vrijgave/storing/sturing). Rick 2026-08-18 + CCA dictionary. Family-agnostic. 7222 manual writes this as DRAK KAB AFG B2CA 3X2X0,8 MT (x32).</t>
   </si>
   <si>
@@ -1547,6 +1541,21 @@
   </si>
   <si>
     <t>rv/&amp;temperatuur</t>
+  </si>
+  <si>
+    <t>POMP_2_SIGNALEN</t>
+  </si>
+  <si>
+    <t>JOBA ST.STR CCCA HCHJZ 7X1 MT</t>
+  </si>
+  <si>
+    <t>JOBA ST.STR cCA HCHJZ 5X1 MT</t>
+  </si>
+  <si>
+    <t>KW_ONLY</t>
+  </si>
+  <si>
+    <t>THE</t>
   </si>
 </sst>
 </file>
@@ -2058,7 +2067,7 @@
         <v>270</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>271</v>
@@ -2072,7 +2081,7 @@
         <v>273</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>274</v>
@@ -2517,7 +2526,7 @@
         <v>49</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="C27" s="3">
         <v>80</v>
@@ -4050,7 +4059,7 @@
     </row>
     <row r="140" spans="1:4">
       <c r="A140" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B140" t="s">
         <v>182</v>
@@ -4064,7 +4073,7 @@
     </row>
     <row r="141" spans="1:4">
       <c r="A141" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="B141" t="s">
         <v>182</v>
@@ -4078,10 +4087,10 @@
     </row>
     <row r="142" spans="1:4">
       <c r="A142" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="B142" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="C142">
         <v>75</v>
@@ -4092,10 +4101,10 @@
     </row>
     <row r="143" spans="1:4">
       <c r="A143" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="B143" s="10" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="C143">
         <v>45</v>
@@ -4106,10 +4115,10 @@
     </row>
     <row r="144" spans="1:4">
       <c r="A144" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="B144" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C144">
         <v>88</v>
@@ -4117,10 +4126,10 @@
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="B145" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C145">
         <v>88</v>
@@ -4133,7 +4142,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -4391,10 +4400,10 @@
         <v>315</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>337</v>
@@ -5057,7 +5066,7 @@
         <v>320</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F48" t="s">
         <v>401</v>
@@ -5105,7 +5114,7 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="B51" t="s">
         <v>318</v>
@@ -5117,7 +5126,7 @@
         <v>320</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F51" t="s">
         <v>404</v>
@@ -5137,7 +5146,7 @@
         <v>320</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>320</v>
+        <v>507</v>
       </c>
       <c r="F52" t="s">
         <v>405</v>
@@ -5153,50 +5162,56 @@
       <c r="C53" t="s">
         <v>363</v>
       </c>
+      <c r="D53" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="54" spans="1:6">
       <c r="A54" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="B54" t="s">
+        <v>318</v>
+      </c>
+      <c r="C54" t="s">
+        <v>319</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="F54" t="s">
         <v>407</v>
-      </c>
-      <c r="C54" t="s">
-        <v>407</v>
-      </c>
-      <c r="D54" t="s">
-        <v>407</v>
-      </c>
-      <c r="E54" t="s">
-        <v>407</v>
-      </c>
-      <c r="F54" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="55" spans="1:6">
       <c r="A55" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="B55" t="s">
-        <v>410</v>
+        <v>342</v>
       </c>
       <c r="C55" t="s">
-        <v>410</v>
-      </c>
-      <c r="D55" t="s">
-        <v>410</v>
-      </c>
-      <c r="E55" t="s">
-        <v>410</v>
+        <v>343</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>335</v>
       </c>
       <c r="F55" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="B56" t="s">
         <v>332</v>
@@ -5213,13 +5228,13 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" t="s">
+        <v>487</v>
+      </c>
+      <c r="B57" t="s">
+        <v>490</v>
+      </c>
+      <c r="C57" t="s">
         <v>489</v>
-      </c>
-      <c r="B57" t="s">
-        <v>492</v>
-      </c>
-      <c r="C57" t="s">
-        <v>491</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>320</v>
@@ -5230,13 +5245,13 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="10" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="B58" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C58" t="s">
-        <v>491</v>
+        <v>509</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>320</v>
@@ -5247,67 +5262,67 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="B59" t="s">
-        <v>407</v>
+        <v>318</v>
       </c>
       <c r="C59" t="s">
-        <v>407</v>
-      </c>
-      <c r="D59" t="s">
-        <v>407</v>
-      </c>
-      <c r="E59" t="s">
-        <v>407</v>
+        <v>319</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>321</v>
       </c>
       <c r="F59" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="B60" t="s">
-        <v>410</v>
+        <v>342</v>
       </c>
       <c r="C60" t="s">
-        <v>410</v>
-      </c>
-      <c r="D60" t="s">
-        <v>410</v>
-      </c>
-      <c r="E60" t="s">
-        <v>410</v>
+        <v>343</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>506</v>
       </c>
       <c r="F60" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="61" spans="1:6">
       <c r="A61" t="s">
+        <v>408</v>
+      </c>
+      <c r="B61" t="s">
+        <v>342</v>
+      </c>
+      <c r="C61" t="s">
+        <v>343</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="F61" t="s">
         <v>409</v>
-      </c>
-      <c r="B61" t="s">
-        <v>410</v>
-      </c>
-      <c r="C61" t="s">
-        <v>410</v>
-      </c>
-      <c r="D61" t="s">
-        <v>410</v>
-      </c>
-      <c r="E61" t="s">
-        <v>410</v>
-      </c>
-      <c r="F61" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B62" t="s">
         <v>327</v>
@@ -5327,7 +5342,7 @@
     </row>
     <row r="63" spans="1:6">
       <c r="A63" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="B63" s="8" t="s">
         <v>391</v>
@@ -5343,6 +5358,26 @@
       </c>
       <c r="F63" t="s">
         <v>403</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" t="s">
+        <v>505</v>
+      </c>
+      <c r="B64" t="s">
+        <v>318</v>
+      </c>
+      <c r="C64" t="s">
+        <v>319</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="F64" t="s">
+        <v>409</v>
       </c>
     </row>
   </sheetData>
@@ -5352,7 +5387,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -5363,41 +5398,41 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="5" t="s">
         <v>416</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="5" t="s">
         <v>417</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>418</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="I3" s="5" t="s">
         <v>419</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>420</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>421</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="3" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>349</v>
@@ -5409,15 +5444,15 @@
         <v>1</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="3" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>370</v>
@@ -5426,12 +5461,12 @@
         <v>1</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="3" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>356</v>
@@ -5443,7 +5478,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -5462,34 +5497,45 @@
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="3" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="3" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>370</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5509,18 +5555,18 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>434</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>436</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>305</v>
@@ -5528,21 +5574,21 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>391</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>391</v>
@@ -5551,12 +5597,12 @@
         <v>281</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>382</v>
@@ -5565,15 +5611,15 @@
         <v>281</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="3" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>281</v>
@@ -5582,21 +5628,21 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="3" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>281</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="3" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="B9" t="s">
         <v>307</v>
@@ -5622,23 +5668,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -5646,71 +5692,71 @@
         <v>98</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="3" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="3" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="3" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="B11" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="B12" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B13" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
   </sheetData>
@@ -5730,64 +5776,64 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="6" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>471</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>472</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B4" t="s">
+        <v>473</v>
+      </c>
+      <c r="C4" t="s">
         <v>474</v>
-      </c>
-      <c r="B4" t="s">
-        <v>475</v>
-      </c>
-      <c r="C4" t="s">
-        <v>476</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="B5" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="C5" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
+        <v>476</v>
+      </c>
+      <c r="B6" t="s">
+        <v>477</v>
+      </c>
+      <c r="C6" t="s">
         <v>478</v>
-      </c>
-      <c r="B6" t="s">
-        <v>479</v>
-      </c>
-      <c r="C6" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="B7" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="B8" t="s">
         <v>289</v>

</xml_diff>